<commit_message>
docs: add GitHub URL to contribution table
</commit_message>
<xml_diff>
--- a/贡献分配表.xlsx
+++ b/贡献分配表.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +32,15 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -66,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -82,6 +91,8 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -447,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -559,7 +570,22 @@
       </c>
       <c r="C7" s="4" t="n"/>
     </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>GitHub 地址</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>https://github.com/Kkkkkkkkkkkkenny/VAST-Challenge-2022-Mini-Challenge-1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B9:C9"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>